<commit_message>
data: 台股 財報估值(179檔, 自算PER) 20260624
</commit_message>
<xml_diff>
--- a/data/20260624_台股財報估值.xlsx
+++ b/data/20260624_台股財報估值.xlsx
@@ -658,7 +658,11 @@
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -834,7 +838,11 @@
       <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="inlineStr"/>
       <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -915,7 +923,11 @@
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1376,7 +1388,11 @@
       <c r="Z10" t="inlineStr"/>
       <c r="AA10" t="inlineStr"/>
       <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1647,7 +1663,11 @@
       <c r="Z13" t="inlineStr"/>
       <c r="AA13" t="inlineStr"/>
       <c r="AB13" t="inlineStr"/>
-      <c r="AC13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2488,7 +2508,11 @@
       <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="inlineStr"/>
       <c r="AB22" t="inlineStr"/>
-      <c r="AC22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2569,7 +2593,11 @@
       <c r="Z23" t="inlineStr"/>
       <c r="AA23" t="inlineStr"/>
       <c r="AB23" t="inlineStr"/>
-      <c r="AC23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2650,7 +2678,11 @@
       <c r="Z24" t="inlineStr"/>
       <c r="AA24" t="inlineStr"/>
       <c r="AB24" t="inlineStr"/>
-      <c r="AC24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2826,7 +2858,11 @@
       <c r="Z26" t="inlineStr"/>
       <c r="AA26" t="inlineStr"/>
       <c r="AB26" t="inlineStr"/>
-      <c r="AC26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2907,7 +2943,11 @@
       <c r="Z27" t="inlineStr"/>
       <c r="AA27" t="inlineStr"/>
       <c r="AB27" t="inlineStr"/>
-      <c r="AC27" t="inlineStr"/>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2988,7 +3028,11 @@
       <c r="Z28" t="inlineStr"/>
       <c r="AA28" t="inlineStr"/>
       <c r="AB28" t="inlineStr"/>
-      <c r="AC28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3259,7 +3303,11 @@
       <c r="Z31" t="inlineStr"/>
       <c r="AA31" t="inlineStr"/>
       <c r="AB31" t="inlineStr"/>
-      <c r="AC31" t="inlineStr"/>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3430,22 +3478,14 @@
       <c r="W33" t="n">
         <v>17.5</v>
       </c>
-      <c r="X33" t="n">
-        <v>-2.6</v>
-      </c>
-      <c r="Y33" t="n">
-        <v>12.44</v>
-      </c>
-      <c r="Z33" t="n">
-        <v>26.8</v>
-      </c>
-      <c r="AA33" t="n">
-        <v>26.8</v>
-      </c>
+      <c r="X33" t="inlineStr"/>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="inlineStr"/>
       <c r="AB33" t="inlineStr"/>
       <c r="AC33" t="inlineStr">
         <is>
-          <t>🟠未來偏貴</t>
+          <t>⏸ 成長為負(-3%)</t>
         </is>
       </c>
     </row>
@@ -3623,7 +3663,11 @@
       <c r="Z35" t="inlineStr"/>
       <c r="AA35" t="inlineStr"/>
       <c r="AB35" t="inlineStr"/>
-      <c r="AC35" t="inlineStr"/>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3799,7 +3843,11 @@
       <c r="Z37" t="inlineStr"/>
       <c r="AA37" t="inlineStr"/>
       <c r="AB37" t="inlineStr"/>
-      <c r="AC37" t="inlineStr"/>
+      <c r="AC37" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3880,7 +3928,11 @@
       <c r="Z38" t="inlineStr"/>
       <c r="AA38" t="inlineStr"/>
       <c r="AB38" t="inlineStr"/>
-      <c r="AC38" t="inlineStr"/>
+      <c r="AC38" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3961,7 +4013,11 @@
       <c r="Z39" t="inlineStr"/>
       <c r="AA39" t="inlineStr"/>
       <c r="AB39" t="inlineStr"/>
-      <c r="AC39" t="inlineStr"/>
+      <c r="AC39" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4042,7 +4098,11 @@
       <c r="Z40" t="inlineStr"/>
       <c r="AA40" t="inlineStr"/>
       <c r="AB40" t="inlineStr"/>
-      <c r="AC40" t="inlineStr"/>
+      <c r="AC40" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4218,7 +4278,11 @@
       <c r="Z42" t="inlineStr"/>
       <c r="AA42" t="inlineStr"/>
       <c r="AB42" t="inlineStr"/>
-      <c r="AC42" t="inlineStr"/>
+      <c r="AC42" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4394,7 +4458,11 @@
       <c r="Z44" t="inlineStr"/>
       <c r="AA44" t="inlineStr"/>
       <c r="AB44" t="inlineStr"/>
-      <c r="AC44" t="inlineStr"/>
+      <c r="AC44" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4470,22 +4538,14 @@
       <c r="W45" t="n">
         <v>32.1</v>
       </c>
-      <c r="X45" t="n">
-        <v>-2.9</v>
-      </c>
-      <c r="Y45" t="n">
-        <v>12.56</v>
-      </c>
-      <c r="Z45" t="n">
-        <v>39.8</v>
-      </c>
-      <c r="AA45" t="n">
-        <v>39.8</v>
-      </c>
+      <c r="X45" t="inlineStr"/>
+      <c r="Y45" t="inlineStr"/>
+      <c r="Z45" t="inlineStr"/>
+      <c r="AA45" t="inlineStr"/>
       <c r="AB45" t="inlineStr"/>
       <c r="AC45" t="inlineStr">
         <is>
-          <t>🔴未來過熱</t>
+          <t>⏸ 成長為負(-3%)</t>
         </is>
       </c>
     </row>
@@ -4663,7 +4723,11 @@
       <c r="Z47" t="inlineStr"/>
       <c r="AA47" t="inlineStr"/>
       <c r="AB47" t="inlineStr"/>
-      <c r="AC47" t="inlineStr"/>
+      <c r="AC47" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4934,7 +4998,11 @@
       <c r="Z50" t="inlineStr"/>
       <c r="AA50" t="inlineStr"/>
       <c r="AB50" t="inlineStr"/>
-      <c r="AC50" t="inlineStr"/>
+      <c r="AC50" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5110,7 +5178,11 @@
       <c r="Z52" t="inlineStr"/>
       <c r="AA52" t="inlineStr"/>
       <c r="AB52" t="inlineStr"/>
-      <c r="AC52" t="inlineStr"/>
+      <c r="AC52" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5286,7 +5358,11 @@
       <c r="Z54" t="inlineStr"/>
       <c r="AA54" t="inlineStr"/>
       <c r="AB54" t="inlineStr"/>
-      <c r="AC54" t="inlineStr"/>
+      <c r="AC54" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5462,7 +5538,11 @@
       <c r="Z56" t="inlineStr"/>
       <c r="AA56" t="inlineStr"/>
       <c r="AB56" t="inlineStr"/>
-      <c r="AC56" t="inlineStr"/>
+      <c r="AC56" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5638,7 +5718,11 @@
       <c r="Z58" t="inlineStr"/>
       <c r="AA58" t="inlineStr"/>
       <c r="AB58" t="inlineStr"/>
-      <c r="AC58" t="inlineStr"/>
+      <c r="AC58" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5814,7 +5898,11 @@
       <c r="Z60" t="inlineStr"/>
       <c r="AA60" t="inlineStr"/>
       <c r="AB60" t="inlineStr"/>
-      <c r="AC60" t="inlineStr"/>
+      <c r="AC60" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6180,7 +6268,11 @@
       <c r="Z64" t="inlineStr"/>
       <c r="AA64" t="inlineStr"/>
       <c r="AB64" t="inlineStr"/>
-      <c r="AC64" t="inlineStr"/>
+      <c r="AC64" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -6261,7 +6353,11 @@
       <c r="Z65" t="inlineStr"/>
       <c r="AA65" t="inlineStr"/>
       <c r="AB65" t="inlineStr"/>
-      <c r="AC65" t="inlineStr"/>
+      <c r="AC65" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -6627,7 +6723,11 @@
       <c r="Z69" t="inlineStr"/>
       <c r="AA69" t="inlineStr"/>
       <c r="AB69" t="inlineStr"/>
-      <c r="AC69" t="inlineStr"/>
+      <c r="AC69" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6803,7 +6903,11 @@
       <c r="Z71" t="inlineStr"/>
       <c r="AA71" t="inlineStr"/>
       <c r="AB71" t="inlineStr"/>
-      <c r="AC71" t="inlineStr"/>
+      <c r="AC71" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6979,7 +7083,11 @@
       <c r="Z73" t="inlineStr"/>
       <c r="AA73" t="inlineStr"/>
       <c r="AB73" t="inlineStr"/>
-      <c r="AC73" t="inlineStr"/>
+      <c r="AC73" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -7060,7 +7168,11 @@
       <c r="Z74" t="inlineStr"/>
       <c r="AA74" t="inlineStr"/>
       <c r="AB74" t="inlineStr"/>
-      <c r="AC74" t="inlineStr"/>
+      <c r="AC74" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -7141,7 +7253,11 @@
       <c r="Z75" t="inlineStr"/>
       <c r="AA75" t="inlineStr"/>
       <c r="AB75" t="inlineStr"/>
-      <c r="AC75" t="inlineStr"/>
+      <c r="AC75" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -7222,7 +7338,11 @@
       <c r="Z76" t="inlineStr"/>
       <c r="AA76" t="inlineStr"/>
       <c r="AB76" t="inlineStr"/>
-      <c r="AC76" t="inlineStr"/>
+      <c r="AC76" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -7398,7 +7518,11 @@
       <c r="Z78" t="inlineStr"/>
       <c r="AA78" t="inlineStr"/>
       <c r="AB78" t="inlineStr"/>
-      <c r="AC78" t="inlineStr"/>
+      <c r="AC78" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7574,7 +7698,11 @@
       <c r="Z80" t="inlineStr"/>
       <c r="AA80" t="inlineStr"/>
       <c r="AB80" t="inlineStr"/>
-      <c r="AC80" t="inlineStr"/>
+      <c r="AC80" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -7655,7 +7783,11 @@
       <c r="Z81" t="inlineStr"/>
       <c r="AA81" t="inlineStr"/>
       <c r="AB81" t="inlineStr"/>
-      <c r="AC81" t="inlineStr"/>
+      <c r="AC81" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -7831,7 +7963,11 @@
       <c r="Z83" t="inlineStr"/>
       <c r="AA83" t="inlineStr"/>
       <c r="AB83" t="inlineStr"/>
-      <c r="AC83" t="inlineStr"/>
+      <c r="AC83" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -8197,7 +8333,11 @@
       <c r="Z87" t="inlineStr"/>
       <c r="AA87" t="inlineStr"/>
       <c r="AB87" t="inlineStr"/>
-      <c r="AC87" t="inlineStr"/>
+      <c r="AC87" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -8278,7 +8418,11 @@
       <c r="Z88" t="inlineStr"/>
       <c r="AA88" t="inlineStr"/>
       <c r="AB88" t="inlineStr"/>
-      <c r="AC88" t="inlineStr"/>
+      <c r="AC88" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -8359,7 +8503,11 @@
       <c r="Z89" t="inlineStr"/>
       <c r="AA89" t="inlineStr"/>
       <c r="AB89" t="inlineStr"/>
-      <c r="AC89" t="inlineStr"/>
+      <c r="AC89" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -8720,22 +8868,14 @@
       <c r="W93" t="n">
         <v>52.1</v>
       </c>
-      <c r="X93" t="n">
-        <v>-9</v>
-      </c>
-      <c r="Y93" t="n">
-        <v>3.94</v>
-      </c>
-      <c r="Z93" t="n">
-        <v>15</v>
-      </c>
-      <c r="AA93" t="n">
-        <v>15</v>
-      </c>
+      <c r="X93" t="inlineStr"/>
+      <c r="Y93" t="inlineStr"/>
+      <c r="Z93" t="inlineStr"/>
+      <c r="AA93" t="inlineStr"/>
       <c r="AB93" t="inlineStr"/>
       <c r="AC93" t="inlineStr">
         <is>
-          <t>🟢未來便宜</t>
+          <t>⏸ 成長為負(-9%)</t>
         </is>
       </c>
     </row>
@@ -8818,7 +8958,11 @@
       <c r="Z94" t="inlineStr"/>
       <c r="AA94" t="inlineStr"/>
       <c r="AB94" t="inlineStr"/>
-      <c r="AC94" t="inlineStr"/>
+      <c r="AC94" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -8899,7 +9043,11 @@
       <c r="Z95" t="inlineStr"/>
       <c r="AA95" t="inlineStr"/>
       <c r="AB95" t="inlineStr"/>
-      <c r="AC95" t="inlineStr"/>
+      <c r="AC95" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -9170,7 +9318,11 @@
       <c r="Z98" t="inlineStr"/>
       <c r="AA98" t="inlineStr"/>
       <c r="AB98" t="inlineStr"/>
-      <c r="AC98" t="inlineStr"/>
+      <c r="AC98" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -9346,7 +9498,11 @@
       <c r="Z100" t="inlineStr"/>
       <c r="AA100" t="inlineStr"/>
       <c r="AB100" t="inlineStr"/>
-      <c r="AC100" t="inlineStr"/>
+      <c r="AC100" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -9522,7 +9678,11 @@
       <c r="Z102" t="inlineStr"/>
       <c r="AA102" t="inlineStr"/>
       <c r="AB102" t="inlineStr"/>
-      <c r="AC102" t="inlineStr"/>
+      <c r="AC102" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -9603,7 +9763,11 @@
       <c r="Z103" t="inlineStr"/>
       <c r="AA103" t="inlineStr"/>
       <c r="AB103" t="inlineStr"/>
-      <c r="AC103" t="inlineStr"/>
+      <c r="AC103" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -9684,7 +9848,11 @@
       <c r="Z104" t="inlineStr"/>
       <c r="AA104" t="inlineStr"/>
       <c r="AB104" t="inlineStr"/>
-      <c r="AC104" t="inlineStr"/>
+      <c r="AC104" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -9765,7 +9933,11 @@
       <c r="Z105" t="inlineStr"/>
       <c r="AA105" t="inlineStr"/>
       <c r="AB105" t="inlineStr"/>
-      <c r="AC105" t="inlineStr"/>
+      <c r="AC105" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -10036,7 +10208,11 @@
       <c r="Z108" t="inlineStr"/>
       <c r="AA108" t="inlineStr"/>
       <c r="AB108" t="inlineStr"/>
-      <c r="AC108" t="inlineStr"/>
+      <c r="AC108" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -10117,7 +10293,11 @@
       <c r="Z109" t="inlineStr"/>
       <c r="AA109" t="inlineStr"/>
       <c r="AB109" t="inlineStr"/>
-      <c r="AC109" t="inlineStr"/>
+      <c r="AC109" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -10198,7 +10378,11 @@
       <c r="Z110" t="inlineStr"/>
       <c r="AA110" t="inlineStr"/>
       <c r="AB110" t="inlineStr"/>
-      <c r="AC110" t="inlineStr"/>
+      <c r="AC110" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -10279,7 +10463,11 @@
       <c r="Z111" t="inlineStr"/>
       <c r="AA111" t="inlineStr"/>
       <c r="AB111" t="inlineStr"/>
-      <c r="AC111" t="inlineStr"/>
+      <c r="AC111" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -10455,7 +10643,11 @@
       <c r="Z113" t="inlineStr"/>
       <c r="AA113" t="inlineStr"/>
       <c r="AB113" t="inlineStr"/>
-      <c r="AC113" t="inlineStr"/>
+      <c r="AC113" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -10721,22 +10913,14 @@
       <c r="W116" t="n">
         <v>30.2</v>
       </c>
-      <c r="X116" t="n">
-        <v>-16.5</v>
-      </c>
-      <c r="Y116" t="n">
-        <v>7.02</v>
-      </c>
-      <c r="Z116" t="n">
-        <v>52.2</v>
-      </c>
-      <c r="AA116" t="n">
-        <v>52.2</v>
-      </c>
+      <c r="X116" t="inlineStr"/>
+      <c r="Y116" t="inlineStr"/>
+      <c r="Z116" t="inlineStr"/>
+      <c r="AA116" t="inlineStr"/>
       <c r="AB116" t="inlineStr"/>
       <c r="AC116" t="inlineStr">
         <is>
-          <t>🔴未來過熱</t>
+          <t>⏸ 成長為負(-16%)</t>
         </is>
       </c>
     </row>
@@ -11009,7 +11193,11 @@
       <c r="Z119" t="inlineStr"/>
       <c r="AA119" t="inlineStr"/>
       <c r="AB119" t="inlineStr"/>
-      <c r="AC119" t="inlineStr"/>
+      <c r="AC119" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -11086,7 +11274,11 @@
       <c r="Z120" t="inlineStr"/>
       <c r="AA120" t="inlineStr"/>
       <c r="AB120" t="inlineStr"/>
-      <c r="AC120" t="inlineStr"/>
+      <c r="AC120" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -11167,7 +11359,11 @@
       <c r="Z121" t="inlineStr"/>
       <c r="AA121" t="inlineStr"/>
       <c r="AB121" t="inlineStr"/>
-      <c r="AC121" t="inlineStr"/>
+      <c r="AC121" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -11248,7 +11444,11 @@
       <c r="Z122" t="inlineStr"/>
       <c r="AA122" t="inlineStr"/>
       <c r="AB122" t="inlineStr"/>
-      <c r="AC122" t="inlineStr"/>
+      <c r="AC122" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -11519,7 +11719,11 @@
       <c r="Z125" t="inlineStr"/>
       <c r="AA125" t="inlineStr"/>
       <c r="AB125" t="inlineStr"/>
-      <c r="AC125" t="inlineStr"/>
+      <c r="AC125" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -11695,7 +11899,11 @@
       <c r="Z127" t="inlineStr"/>
       <c r="AA127" t="inlineStr"/>
       <c r="AB127" t="inlineStr"/>
-      <c r="AC127" t="inlineStr"/>
+      <c r="AC127" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -11776,7 +11984,11 @@
       <c r="Z128" t="inlineStr"/>
       <c r="AA128" t="inlineStr"/>
       <c r="AB128" t="inlineStr"/>
-      <c r="AC128" t="inlineStr"/>
+      <c r="AC128" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -11857,7 +12069,11 @@
       <c r="Z129" t="inlineStr"/>
       <c r="AA129" t="inlineStr"/>
       <c r="AB129" t="inlineStr"/>
-      <c r="AC129" t="inlineStr"/>
+      <c r="AC129" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -12033,7 +12249,11 @@
       <c r="Z131" t="inlineStr"/>
       <c r="AA131" t="inlineStr"/>
       <c r="AB131" t="inlineStr"/>
-      <c r="AC131" t="inlineStr"/>
+      <c r="AC131" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -12299,22 +12519,14 @@
       <c r="W134" t="n">
         <v>22.1</v>
       </c>
-      <c r="X134" t="n">
-        <v>-5.7</v>
-      </c>
-      <c r="Y134" t="n">
-        <v>5.38</v>
-      </c>
-      <c r="Z134" t="n">
-        <v>36</v>
-      </c>
-      <c r="AA134" t="n">
-        <v>36</v>
-      </c>
+      <c r="X134" t="inlineStr"/>
+      <c r="Y134" t="inlineStr"/>
+      <c r="Z134" t="inlineStr"/>
+      <c r="AA134" t="inlineStr"/>
       <c r="AB134" t="inlineStr"/>
       <c r="AC134" t="inlineStr">
         <is>
-          <t>🔴未來過熱</t>
+          <t>⏸ 成長為負(-6%)</t>
         </is>
       </c>
     </row>
@@ -12397,7 +12609,11 @@
       <c r="Z135" t="inlineStr"/>
       <c r="AA135" t="inlineStr"/>
       <c r="AB135" t="inlineStr"/>
-      <c r="AC135" t="inlineStr"/>
+      <c r="AC135" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -12573,7 +12789,11 @@
       <c r="Z137" t="inlineStr"/>
       <c r="AA137" t="inlineStr"/>
       <c r="AB137" t="inlineStr"/>
-      <c r="AC137" t="inlineStr"/>
+      <c r="AC137" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -12654,7 +12874,11 @@
       <c r="Z138" t="inlineStr"/>
       <c r="AA138" t="inlineStr"/>
       <c r="AB138" t="inlineStr"/>
-      <c r="AC138" t="inlineStr"/>
+      <c r="AC138" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -12735,7 +12959,11 @@
       <c r="Z139" t="inlineStr"/>
       <c r="AA139" t="inlineStr"/>
       <c r="AB139" t="inlineStr"/>
-      <c r="AC139" t="inlineStr"/>
+      <c r="AC139" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -12816,7 +13044,11 @@
       <c r="Z140" t="inlineStr"/>
       <c r="AA140" t="inlineStr"/>
       <c r="AB140" t="inlineStr"/>
-      <c r="AC140" t="inlineStr"/>
+      <c r="AC140" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -12897,7 +13129,11 @@
       <c r="Z141" t="inlineStr"/>
       <c r="AA141" t="inlineStr"/>
       <c r="AB141" t="inlineStr"/>
-      <c r="AC141" t="inlineStr"/>
+      <c r="AC141" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -12978,7 +13214,11 @@
       <c r="Z142" t="inlineStr"/>
       <c r="AA142" t="inlineStr"/>
       <c r="AB142" t="inlineStr"/>
-      <c r="AC142" t="inlineStr"/>
+      <c r="AC142" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -13059,7 +13299,11 @@
       <c r="Z143" t="inlineStr"/>
       <c r="AA143" t="inlineStr"/>
       <c r="AB143" t="inlineStr"/>
-      <c r="AC143" t="inlineStr"/>
+      <c r="AC143" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -13140,7 +13384,11 @@
       <c r="Z144" t="inlineStr"/>
       <c r="AA144" t="inlineStr"/>
       <c r="AB144" t="inlineStr"/>
-      <c r="AC144" t="inlineStr"/>
+      <c r="AC144" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -13221,7 +13469,11 @@
       <c r="Z145" t="inlineStr"/>
       <c r="AA145" t="inlineStr"/>
       <c r="AB145" t="inlineStr"/>
-      <c r="AC145" t="inlineStr"/>
+      <c r="AC145" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -13302,7 +13554,11 @@
       <c r="Z146" t="inlineStr"/>
       <c r="AA146" t="inlineStr"/>
       <c r="AB146" t="inlineStr"/>
-      <c r="AC146" t="inlineStr"/>
+      <c r="AC146" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -13383,7 +13639,11 @@
       <c r="Z147" t="inlineStr"/>
       <c r="AA147" t="inlineStr"/>
       <c r="AB147" t="inlineStr"/>
-      <c r="AC147" t="inlineStr"/>
+      <c r="AC147" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -13654,7 +13914,11 @@
       <c r="Z150" t="inlineStr"/>
       <c r="AA150" t="inlineStr"/>
       <c r="AB150" t="inlineStr"/>
-      <c r="AC150" t="inlineStr"/>
+      <c r="AC150" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -13735,7 +13999,11 @@
       <c r="Z151" t="inlineStr"/>
       <c r="AA151" t="inlineStr"/>
       <c r="AB151" t="inlineStr"/>
-      <c r="AC151" t="inlineStr"/>
+      <c r="AC151" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -13911,7 +14179,11 @@
       <c r="Z153" t="inlineStr"/>
       <c r="AA153" t="inlineStr"/>
       <c r="AB153" t="inlineStr"/>
-      <c r="AC153" t="inlineStr"/>
+      <c r="AC153" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -13986,7 +14258,11 @@
       <c r="Z154" t="inlineStr"/>
       <c r="AA154" t="inlineStr"/>
       <c r="AB154" t="inlineStr"/>
-      <c r="AC154" t="inlineStr"/>
+      <c r="AC154" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -14067,7 +14343,11 @@
       <c r="Z155" t="inlineStr"/>
       <c r="AA155" t="inlineStr"/>
       <c r="AB155" t="inlineStr"/>
-      <c r="AC155" t="inlineStr"/>
+      <c r="AC155" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -14243,7 +14523,11 @@
       <c r="Z157" t="inlineStr"/>
       <c r="AA157" t="inlineStr"/>
       <c r="AB157" t="inlineStr"/>
-      <c r="AC157" t="inlineStr"/>
+      <c r="AC157" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -14324,7 +14608,11 @@
       <c r="Z158" t="inlineStr"/>
       <c r="AA158" t="inlineStr"/>
       <c r="AB158" t="inlineStr"/>
-      <c r="AC158" t="inlineStr"/>
+      <c r="AC158" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -14405,7 +14693,11 @@
       <c r="Z159" t="inlineStr"/>
       <c r="AA159" t="inlineStr"/>
       <c r="AB159" t="inlineStr"/>
-      <c r="AC159" t="inlineStr"/>
+      <c r="AC159" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -14581,7 +14873,11 @@
       <c r="Z161" t="inlineStr"/>
       <c r="AA161" t="inlineStr"/>
       <c r="AB161" t="inlineStr"/>
-      <c r="AC161" t="inlineStr"/>
+      <c r="AC161" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -14662,7 +14958,11 @@
       <c r="Z162" t="inlineStr"/>
       <c r="AA162" t="inlineStr"/>
       <c r="AB162" t="inlineStr"/>
-      <c r="AC162" t="inlineStr"/>
+      <c r="AC162" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -14737,7 +15037,11 @@
       <c r="Z163" t="inlineStr"/>
       <c r="AA163" t="inlineStr"/>
       <c r="AB163" t="inlineStr"/>
-      <c r="AC163" t="inlineStr"/>
+      <c r="AC163" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -14818,7 +15122,11 @@
       <c r="Z164" t="inlineStr"/>
       <c r="AA164" t="inlineStr"/>
       <c r="AB164" t="inlineStr"/>
-      <c r="AC164" t="inlineStr"/>
+      <c r="AC164" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -14899,7 +15207,11 @@
       <c r="Z165" t="inlineStr"/>
       <c r="AA165" t="inlineStr"/>
       <c r="AB165" t="inlineStr"/>
-      <c r="AC165" t="inlineStr"/>
+      <c r="AC165" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -14980,7 +15292,11 @@
       <c r="Z166" t="inlineStr"/>
       <c r="AA166" t="inlineStr"/>
       <c r="AB166" t="inlineStr"/>
-      <c r="AC166" t="inlineStr"/>
+      <c r="AC166" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -15061,7 +15377,11 @@
       <c r="Z167" t="inlineStr"/>
       <c r="AA167" t="inlineStr"/>
       <c r="AB167" t="inlineStr"/>
-      <c r="AC167" t="inlineStr"/>
+      <c r="AC167" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -15237,7 +15557,11 @@
       <c r="Z169" t="inlineStr"/>
       <c r="AA169" t="inlineStr"/>
       <c r="AB169" t="inlineStr"/>
-      <c r="AC169" t="inlineStr"/>
+      <c r="AC169" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -15318,7 +15642,11 @@
       <c r="Z170" t="inlineStr"/>
       <c r="AA170" t="inlineStr"/>
       <c r="AB170" t="inlineStr"/>
-      <c r="AC170" t="inlineStr"/>
+      <c r="AC170" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -15399,7 +15727,11 @@
       <c r="Z171" t="inlineStr"/>
       <c r="AA171" t="inlineStr"/>
       <c r="AB171" t="inlineStr"/>
-      <c r="AC171" t="inlineStr"/>
+      <c r="AC171" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -15575,7 +15907,11 @@
       <c r="Z173" t="inlineStr"/>
       <c r="AA173" t="inlineStr"/>
       <c r="AB173" t="inlineStr"/>
-      <c r="AC173" t="inlineStr"/>
+      <c r="AC173" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -15656,7 +15992,11 @@
       <c r="Z174" t="inlineStr"/>
       <c r="AA174" t="inlineStr"/>
       <c r="AB174" t="inlineStr"/>
-      <c r="AC174" t="inlineStr"/>
+      <c r="AC174" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -15737,7 +16077,11 @@
       <c r="Z175" t="inlineStr"/>
       <c r="AA175" t="inlineStr"/>
       <c r="AB175" t="inlineStr"/>
-      <c r="AC175" t="inlineStr"/>
+      <c r="AC175" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -15818,7 +16162,11 @@
       <c r="Z176" t="inlineStr"/>
       <c r="AA176" t="inlineStr"/>
       <c r="AB176" t="inlineStr"/>
-      <c r="AC176" t="inlineStr"/>
+      <c r="AC176" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -15899,7 +16247,11 @@
       <c r="Z177" t="inlineStr"/>
       <c r="AA177" t="inlineStr"/>
       <c r="AB177" t="inlineStr"/>
-      <c r="AC177" t="inlineStr"/>
+      <c r="AC177" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -15980,7 +16332,11 @@
       <c r="Z178" t="inlineStr"/>
       <c r="AA178" t="inlineStr"/>
       <c r="AB178" t="inlineStr"/>
-      <c r="AC178" t="inlineStr"/>
+      <c r="AC178" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -16061,7 +16417,11 @@
       <c r="Z179" t="inlineStr"/>
       <c r="AA179" t="inlineStr"/>
       <c r="AB179" t="inlineStr"/>
-      <c r="AC179" t="inlineStr"/>
+      <c r="AC179" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -16332,7 +16692,11 @@
       <c r="Z182" t="inlineStr"/>
       <c r="AA182" t="inlineStr"/>
       <c r="AB182" t="inlineStr"/>
-      <c r="AC182" t="inlineStr"/>
+      <c r="AC182" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -16413,7 +16777,11 @@
       <c r="Z183" t="inlineStr"/>
       <c r="AA183" t="inlineStr"/>
       <c r="AB183" t="inlineStr"/>
-      <c r="AC183" t="inlineStr"/>
+      <c r="AC183" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -16494,7 +16862,11 @@
       <c r="Z184" t="inlineStr"/>
       <c r="AA184" t="inlineStr"/>
       <c r="AB184" t="inlineStr"/>
-      <c r="AC184" t="inlineStr"/>
+      <c r="AC184" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -16575,7 +16947,11 @@
       <c r="Z185" t="inlineStr"/>
       <c r="AA185" t="inlineStr"/>
       <c r="AB185" t="inlineStr"/>
-      <c r="AC185" t="inlineStr"/>
+      <c r="AC185" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -16656,7 +17032,11 @@
       <c r="Z186" t="inlineStr"/>
       <c r="AA186" t="inlineStr"/>
       <c r="AB186" t="inlineStr"/>
-      <c r="AC186" t="inlineStr"/>
+      <c r="AC186" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -16737,7 +17117,11 @@
       <c r="Z187" t="inlineStr"/>
       <c r="AA187" t="inlineStr"/>
       <c r="AB187" t="inlineStr"/>
-      <c r="AC187" t="inlineStr"/>
+      <c r="AC187" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -16818,7 +17202,11 @@
       <c r="Z188" t="inlineStr"/>
       <c r="AA188" t="inlineStr"/>
       <c r="AB188" t="inlineStr"/>
-      <c r="AC188" t="inlineStr"/>
+      <c r="AC188" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -16899,7 +17287,11 @@
       <c r="Z189" t="inlineStr"/>
       <c r="AA189" t="inlineStr"/>
       <c r="AB189" t="inlineStr"/>
-      <c r="AC189" t="inlineStr"/>
+      <c r="AC189" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -16980,7 +17372,11 @@
       <c r="Z190" t="inlineStr"/>
       <c r="AA190" t="inlineStr"/>
       <c r="AB190" t="inlineStr"/>
-      <c r="AC190" t="inlineStr"/>
+      <c r="AC190" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -17138,7 +17534,11 @@
       <c r="Z192" t="inlineStr"/>
       <c r="AA192" t="inlineStr"/>
       <c r="AB192" t="inlineStr"/>
-      <c r="AC192" t="inlineStr"/>
+      <c r="AC192" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -17219,7 +17619,11 @@
       <c r="Z193" t="inlineStr"/>
       <c r="AA193" t="inlineStr"/>
       <c r="AB193" t="inlineStr"/>
-      <c r="AC193" t="inlineStr"/>
+      <c r="AC193" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -17300,7 +17704,11 @@
       <c r="Z194" t="inlineStr"/>
       <c r="AA194" t="inlineStr"/>
       <c r="AB194" t="inlineStr"/>
-      <c r="AC194" t="inlineStr"/>
+      <c r="AC194" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -17381,7 +17789,11 @@
       <c r="Z195" t="inlineStr"/>
       <c r="AA195" t="inlineStr"/>
       <c r="AB195" t="inlineStr"/>
-      <c r="AC195" t="inlineStr"/>
+      <c r="AC195" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -17462,7 +17874,11 @@
       <c r="Z196" t="inlineStr"/>
       <c r="AA196" t="inlineStr"/>
       <c r="AB196" t="inlineStr"/>
-      <c r="AC196" t="inlineStr"/>
+      <c r="AC196" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -17543,7 +17959,11 @@
       <c r="Z197" t="inlineStr"/>
       <c r="AA197" t="inlineStr"/>
       <c r="AB197" t="inlineStr"/>
-      <c r="AC197" t="inlineStr"/>
+      <c r="AC197" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -17624,7 +18044,11 @@
       <c r="Z198" t="inlineStr"/>
       <c r="AA198" t="inlineStr"/>
       <c r="AB198" t="inlineStr"/>
-      <c r="AC198" t="inlineStr"/>
+      <c r="AC198" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -17705,7 +18129,11 @@
       <c r="Z199" t="inlineStr"/>
       <c r="AA199" t="inlineStr"/>
       <c r="AB199" t="inlineStr"/>
-      <c r="AC199" t="inlineStr"/>
+      <c r="AC199" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -17786,7 +18214,11 @@
       <c r="Z200" t="inlineStr"/>
       <c r="AA200" t="inlineStr"/>
       <c r="AB200" t="inlineStr"/>
-      <c r="AC200" t="inlineStr"/>
+      <c r="AC200" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -17867,7 +18299,11 @@
       <c r="Z201" t="inlineStr"/>
       <c r="AA201" t="inlineStr"/>
       <c r="AB201" t="inlineStr"/>
-      <c r="AC201" t="inlineStr"/>
+      <c r="AC201" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -17948,7 +18384,11 @@
       <c r="Z202" t="inlineStr"/>
       <c r="AA202" t="inlineStr"/>
       <c r="AB202" t="inlineStr"/>
-      <c r="AC202" t="inlineStr"/>
+      <c r="AC202" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -18029,7 +18469,11 @@
       <c r="Z203" t="inlineStr"/>
       <c r="AA203" t="inlineStr"/>
       <c r="AB203" t="inlineStr"/>
-      <c r="AC203" t="inlineStr"/>
+      <c r="AC203" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -18110,7 +18554,11 @@
       <c r="Z204" t="inlineStr"/>
       <c r="AA204" t="inlineStr"/>
       <c r="AB204" t="inlineStr"/>
-      <c r="AC204" t="inlineStr"/>
+      <c r="AC204" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -18191,7 +18639,11 @@
       <c r="Z205" t="inlineStr"/>
       <c r="AA205" t="inlineStr"/>
       <c r="AB205" t="inlineStr"/>
-      <c r="AC205" t="inlineStr"/>
+      <c r="AC205" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -18272,7 +18724,11 @@
       <c r="Z206" t="inlineStr"/>
       <c r="AA206" t="inlineStr"/>
       <c r="AB206" t="inlineStr"/>
-      <c r="AC206" t="inlineStr"/>
+      <c r="AC206" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -18353,7 +18809,11 @@
       <c r="Z207" t="inlineStr"/>
       <c r="AA207" t="inlineStr"/>
       <c r="AB207" t="inlineStr"/>
-      <c r="AC207" t="inlineStr"/>
+      <c r="AC207" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -18434,7 +18894,11 @@
       <c r="Z208" t="inlineStr"/>
       <c r="AA208" t="inlineStr"/>
       <c r="AB208" t="inlineStr"/>
-      <c r="AC208" t="inlineStr"/>
+      <c r="AC208" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -18515,7 +18979,11 @@
       <c r="Z209" t="inlineStr"/>
       <c r="AA209" t="inlineStr"/>
       <c r="AB209" t="inlineStr"/>
-      <c r="AC209" t="inlineStr"/>
+      <c r="AC209" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -18691,7 +19159,11 @@
       <c r="Z211" t="inlineStr"/>
       <c r="AA211" t="inlineStr"/>
       <c r="AB211" t="inlineStr"/>
-      <c r="AC211" t="inlineStr"/>
+      <c r="AC211" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -18772,7 +19244,11 @@
       <c r="Z212" t="inlineStr"/>
       <c r="AA212" t="inlineStr"/>
       <c r="AB212" t="inlineStr"/>
-      <c r="AC212" t="inlineStr"/>
+      <c r="AC212" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -18853,7 +19329,11 @@
       <c r="Z213" t="inlineStr"/>
       <c r="AA213" t="inlineStr"/>
       <c r="AB213" t="inlineStr"/>
-      <c r="AC213" t="inlineStr"/>
+      <c r="AC213" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -18934,7 +19414,11 @@
       <c r="Z214" t="inlineStr"/>
       <c r="AA214" t="inlineStr"/>
       <c r="AB214" t="inlineStr"/>
-      <c r="AC214" t="inlineStr"/>
+      <c r="AC214" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -19015,7 +19499,11 @@
       <c r="Z215" t="inlineStr"/>
       <c r="AA215" t="inlineStr"/>
       <c r="AB215" t="inlineStr"/>
-      <c r="AC215" t="inlineStr"/>
+      <c r="AC215" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -19096,7 +19584,11 @@
       <c r="Z216" t="inlineStr"/>
       <c r="AA216" t="inlineStr"/>
       <c r="AB216" t="inlineStr"/>
-      <c r="AC216" t="inlineStr"/>
+      <c r="AC216" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -19177,7 +19669,11 @@
       <c r="Z217" t="inlineStr"/>
       <c r="AA217" t="inlineStr"/>
       <c r="AB217" t="inlineStr"/>
-      <c r="AC217" t="inlineStr"/>
+      <c r="AC217" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -19248,7 +19744,11 @@
       <c r="Z218" t="inlineStr"/>
       <c r="AA218" t="inlineStr"/>
       <c r="AB218" t="inlineStr"/>
-      <c r="AC218" t="inlineStr"/>
+      <c r="AC218" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -19319,7 +19819,11 @@
       <c r="Z219" t="inlineStr"/>
       <c r="AA219" t="inlineStr"/>
       <c r="AB219" t="inlineStr"/>
-      <c r="AC219" t="inlineStr"/>
+      <c r="AC219" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -19475,7 +19979,11 @@
       <c r="Z221" t="inlineStr"/>
       <c r="AA221" t="inlineStr"/>
       <c r="AB221" t="inlineStr"/>
-      <c r="AC221" t="inlineStr"/>
+      <c r="AC221" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -19716,7 +20224,11 @@
       <c r="Z224" t="inlineStr"/>
       <c r="AA224" t="inlineStr"/>
       <c r="AB224" t="inlineStr"/>
-      <c r="AC224" t="inlineStr"/>
+      <c r="AC224" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -19787,7 +20299,11 @@
       <c r="Z225" t="inlineStr"/>
       <c r="AA225" t="inlineStr"/>
       <c r="AB225" t="inlineStr"/>
-      <c r="AC225" t="inlineStr"/>
+      <c r="AC225" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -19858,7 +20374,11 @@
       <c r="Z226" t="inlineStr"/>
       <c r="AA226" t="inlineStr"/>
       <c r="AB226" t="inlineStr"/>
-      <c r="AC226" t="inlineStr"/>
+      <c r="AC226" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -19929,7 +20449,11 @@
       <c r="Z227" t="inlineStr"/>
       <c r="AA227" t="inlineStr"/>
       <c r="AB227" t="inlineStr"/>
-      <c r="AC227" t="inlineStr"/>
+      <c r="AC227" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -20000,7 +20524,11 @@
       <c r="Z228" t="inlineStr"/>
       <c r="AA228" t="inlineStr"/>
       <c r="AB228" t="inlineStr"/>
-      <c r="AC228" t="inlineStr"/>
+      <c r="AC228" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -20081,7 +20609,11 @@
       <c r="Z229" t="inlineStr"/>
       <c r="AA229" t="inlineStr"/>
       <c r="AB229" t="inlineStr"/>
-      <c r="AC229" t="inlineStr"/>
+      <c r="AC229" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -20162,7 +20694,11 @@
       <c r="Z230" t="inlineStr"/>
       <c r="AA230" t="inlineStr"/>
       <c r="AB230" t="inlineStr"/>
-      <c r="AC230" t="inlineStr"/>
+      <c r="AC230" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -20243,7 +20779,11 @@
       <c r="Z231" t="inlineStr"/>
       <c r="AA231" t="inlineStr"/>
       <c r="AB231" t="inlineStr"/>
-      <c r="AC231" t="inlineStr"/>
+      <c r="AC231" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -20324,7 +20864,11 @@
       <c r="Z232" t="inlineStr"/>
       <c r="AA232" t="inlineStr"/>
       <c r="AB232" t="inlineStr"/>
-      <c r="AC232" t="inlineStr"/>
+      <c r="AC232" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -20405,7 +20949,11 @@
       <c r="Z233" t="inlineStr"/>
       <c r="AA233" t="inlineStr"/>
       <c r="AB233" t="inlineStr"/>
-      <c r="AC233" t="inlineStr"/>
+      <c r="AC233" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -20486,7 +21034,11 @@
       <c r="Z234" t="inlineStr"/>
       <c r="AA234" t="inlineStr"/>
       <c r="AB234" t="inlineStr"/>
-      <c r="AC234" t="inlineStr"/>
+      <c r="AC234" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -20567,7 +21119,11 @@
       <c r="Z235" t="inlineStr"/>
       <c r="AA235" t="inlineStr"/>
       <c r="AB235" t="inlineStr"/>
-      <c r="AC235" t="inlineStr"/>
+      <c r="AC235" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -20648,7 +21204,11 @@
       <c r="Z236" t="inlineStr"/>
       <c r="AA236" t="inlineStr"/>
       <c r="AB236" t="inlineStr"/>
-      <c r="AC236" t="inlineStr"/>
+      <c r="AC236" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -20729,7 +21289,11 @@
       <c r="Z237" t="inlineStr"/>
       <c r="AA237" t="inlineStr"/>
       <c r="AB237" t="inlineStr"/>
-      <c r="AC237" t="inlineStr"/>
+      <c r="AC237" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -20802,7 +21366,11 @@
       <c r="Z238" t="inlineStr"/>
       <c r="AA238" t="inlineStr"/>
       <c r="AB238" t="inlineStr"/>
-      <c r="AC238" t="inlineStr"/>
+      <c r="AC238" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -20873,7 +21441,11 @@
       <c r="Z239" t="inlineStr"/>
       <c r="AA239" t="inlineStr"/>
       <c r="AB239" t="inlineStr"/>
-      <c r="AC239" t="inlineStr"/>
+      <c r="AC239" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -20954,7 +21526,11 @@
       <c r="Z240" t="inlineStr"/>
       <c r="AA240" t="inlineStr"/>
       <c r="AB240" t="inlineStr"/>
-      <c r="AC240" t="inlineStr"/>
+      <c r="AC240" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -21027,7 +21603,11 @@
       <c r="Z241" t="inlineStr"/>
       <c r="AA241" t="inlineStr"/>
       <c r="AB241" t="inlineStr"/>
-      <c r="AC241" t="inlineStr"/>
+      <c r="AC241" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -21100,7 +21680,11 @@
       <c r="Z242" t="inlineStr"/>
       <c r="AA242" t="inlineStr"/>
       <c r="AB242" t="inlineStr"/>
-      <c r="AC242" t="inlineStr"/>
+      <c r="AC242" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -21181,7 +21765,11 @@
       <c r="Z243" t="inlineStr"/>
       <c r="AA243" t="inlineStr"/>
       <c r="AB243" t="inlineStr"/>
-      <c r="AC243" t="inlineStr"/>
+      <c r="AC243" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">

</xml_diff>